<commit_message>
Uploaded Springer_Hybrid_scifreeimport.xlsx,  Springer_Nature_Hybrid_OpenChoice.scifreeimport.xlsx,  Springer_Open_scifreeimport.xlsx 260624
</commit_message>
<xml_diff>
--- a/UK_CoP_TitleLists/Springer_Nature_Hybrid_OpenChoice.scifreeimport.xlsx
+++ b/UK_CoP_TitleLists/Springer_Nature_Hybrid_OpenChoice.scifreeimport.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://computingservices-my.sharepoint.com/personal/lc2792_bath_ac_uk/Documents/Documents/SciFree/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9d4b02a2393526de/Documents/CoP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="230" documentId="8_{B5AC4299-6A25-40E0-8620-1B756A641782}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D4E69898-8388-4A39-86FB-C2F2B57757EF}"/>
+  <xr:revisionPtr revIDLastSave="264" documentId="8_{B5AC4299-6A25-40E0-8620-1B756A641782}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C64000DE-D1E5-4EDC-B4FB-F87A722F3DDB}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{BE44926E-75A4-4EDC-A463-0127E7F3749D}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{BE44926E-75A4-4EDC-A463-0127E7F3749D}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal List" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="174">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="344" uniqueCount="172">
   <si>
     <t>Journal Title</t>
   </si>
@@ -133,36 +133,9 @@
     <t>Change Type (See Terms)</t>
   </si>
   <si>
-    <t>0123-4566</t>
-  </si>
-  <si>
-    <t>0123-4567</t>
-  </si>
-  <si>
-    <t>https://www.scifree.se</t>
-  </si>
-  <si>
     <t>Hybrid</t>
   </si>
   <si>
-    <t>CC-BY</t>
-  </si>
-  <si>
-    <t>Example Publisher Name</t>
-  </si>
-  <si>
-    <t>EXAMPLE Journal title</t>
-  </si>
-  <si>
-    <t xml:space="preserve">E.g. Publisher/Imprint, URL, </t>
-  </si>
-  <si>
-    <t xml:space="preserve">E.g. add new publisher name, add new url, </t>
-  </si>
-  <si>
-    <t>History, Visual Arts and Performing Arts</t>
-  </si>
-  <si>
     <t>Not Accepting Submissions</t>
   </si>
   <si>
@@ -442,9 +415,6 @@
     <t>CC BY</t>
   </si>
   <si>
-    <t>Hybrid (Open Choice)</t>
-  </si>
-  <si>
     <t>https://link.springer.com/journal/41586</t>
   </si>
   <si>
@@ -560,13 +530,37 @@
   </si>
   <si>
     <t>https://link.springer.com/journal/44221</t>
+  </si>
+  <si>
+    <t>3005-0693</t>
+  </si>
+  <si>
+    <t>3059-4499</t>
+  </si>
+  <si>
+    <t>Nature Sensors</t>
+  </si>
+  <si>
+    <t>Nature Health</t>
+  </si>
+  <si>
+    <t>Chemistry and Materials Science</t>
+  </si>
+  <si>
+    <t>Medicine &amp; Public Health</t>
+  </si>
+  <si>
+    <t>https://www.nature.com/naturehealth/</t>
+  </si>
+  <si>
+    <t>https://www.nature.com/natsensors/</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="13" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -599,13 +593,6 @@
       <family val="2"/>
     </font>
     <font>
-      <i/>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
       <u/>
       <sz val="11"/>
       <color theme="10"/>
@@ -627,13 +614,6 @@
       <family val="2"/>
     </font>
     <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
       <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -648,6 +628,13 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -780,237 +767,120 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="35">
+  <dxfs count="37">
     <dxf>
       <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color auto="1"/>
-        <name val="Calibri"/>
-        <scheme val="none"/>
+        <color rgb="FF9C0006"/>
       </font>
       <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color theme="9" tint="-0.499984740745262"/>
-        </left>
-        <right style="thin">
-          <color theme="9" tint="-0.499984740745262"/>
-        </right>
-        <top style="thin">
-          <color theme="9" tint="-0.499984740745262"/>
-        </top>
-        <bottom style="thin">
-          <color theme="9" tint="-0.499984740745262"/>
-        </bottom>
-      </border>
     </dxf>
     <dxf>
       <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color auto="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
+        <color rgb="FF9C0006"/>
       </font>
       <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color theme="9" tint="-0.499984740745262"/>
-        </left>
-        <right style="thin">
-          <color theme="9" tint="-0.499984740745262"/>
-        </right>
-        <top style="thin">
-          <color theme="9" tint="-0.499984740745262"/>
-        </top>
-        <bottom style="thin">
-          <color theme="9" tint="-0.499984740745262"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color auto="1"/>
-        <name val="Calibri"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color theme="9" tint="-0.499984740745262"/>
-        </left>
-        <right/>
-        <top style="thin">
-          <color theme="9" tint="-0.499984740745262"/>
-        </top>
-        <bottom style="thin">
-          <color theme="9" tint="-0.499984740745262"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color auto="1"/>
-        <name val="Calibri"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color theme="9" tint="-0.499984740745262"/>
-        </left>
-        <right style="thin">
-          <color theme="9" tint="-0.499984740745262"/>
-        </right>
-        <top style="thin">
-          <color theme="9" tint="-0.499984740745262"/>
-        </top>
-        <bottom style="thin">
-          <color theme="9" tint="-0.499984740745262"/>
-        </bottom>
-      </border>
     </dxf>
     <dxf>
       <font>
@@ -1649,6 +1519,119 @@
         <sz val="12"/>
         <color auto="1"/>
         <name val="Calibri"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color theme="9" tint="-0.499984740745262"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color theme="9" tint="-0.499984740745262"/>
+        </top>
+        <bottom style="thin">
+          <color theme="9" tint="-0.499984740745262"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color theme="9" tint="-0.499984740745262"/>
+        </left>
+        <right style="thin">
+          <color theme="9" tint="-0.499984740745262"/>
+        </right>
+        <top style="thin">
+          <color theme="9" tint="-0.499984740745262"/>
+        </top>
+        <bottom style="thin">
+          <color theme="9" tint="-0.499984740745262"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color theme="9" tint="-0.499984740745262"/>
+        </left>
+        <right style="thin">
+          <color theme="9" tint="-0.499984740745262"/>
+        </right>
+        <top style="thin">
+          <color theme="9" tint="-0.499984740745262"/>
+        </top>
+        <bottom style="thin">
+          <color theme="9" tint="-0.499984740745262"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
         <family val="2"/>
         <scheme val="none"/>
       </font>
@@ -1659,6 +1642,44 @@
         </patternFill>
       </fill>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color theme="9" tint="-0.499984740745262"/>
+        </left>
+        <right style="thin">
+          <color theme="9" tint="-0.499984740745262"/>
+        </right>
+        <top style="thin">
+          <color theme="9" tint="-0.499984740745262"/>
+        </top>
+        <bottom style="thin">
+          <color theme="9" tint="-0.499984740745262"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color theme="9" tint="-0.499984740745262"/>
@@ -1898,51 +1919,55 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4E20557D-7D01-4DDD-A3E5-4BE8969774E1}" name="Table1" displayName="Table1" ref="A1:H40" totalsRowShown="0" headerRowDxfId="34" dataDxfId="32" headerRowBorderDxfId="33" tableBorderDxfId="31" totalsRowBorderDxfId="30">
-  <autoFilter ref="A1:H40" xr:uid="{4E20557D-7D01-4DDD-A3E5-4BE8969774E1}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4E20557D-7D01-4DDD-A3E5-4BE8969774E1}" name="Table1" displayName="Table1" ref="A1:H42" totalsRowShown="0" headerRowDxfId="36" dataDxfId="34" headerRowBorderDxfId="35" tableBorderDxfId="33" totalsRowBorderDxfId="32">
+  <autoFilter ref="A1:H42" xr:uid="{4E20557D-7D01-4DDD-A3E5-4BE8969774E1}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{60C9D913-7610-4E89-96C3-79D540E13C81}" name="Journal Title" dataDxfId="29"/>
-    <tableColumn id="2" xr3:uid="{157A6765-6BEB-45C8-B059-14466701E200}" name="Imprint" dataDxfId="28"/>
-    <tableColumn id="3" xr3:uid="{C2D0AE15-8EB6-42FA-9756-6359A70C39F2}" name="Print ISSN" dataDxfId="27"/>
-    <tableColumn id="4" xr3:uid="{C1A14781-2EC2-4655-8B99-34C639B681F7}" name="Electronic ISSN" dataDxfId="3"/>
-    <tableColumn id="5" xr3:uid="{6A1CDB50-05D6-4137-BED6-66AEA762C1D8}" name="Journal URL" dataDxfId="26"/>
-    <tableColumn id="6" xr3:uid="{142F869A-41EF-4110-B212-DCDFE3A91B4D}" name="Publishing Model" dataDxfId="0"/>
-    <tableColumn id="7" xr3:uid="{883DC121-F62A-4717-ABC9-50C24089DAAE}" name="License Options" dataDxfId="1"/>
-    <tableColumn id="8" xr3:uid="{79ADE6AD-15D5-4E9E-ADB0-716C42F18B23}" name="Subject Areas" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{60C9D913-7610-4E89-96C3-79D540E13C81}" name="Journal Title" dataDxfId="31"/>
+    <tableColumn id="2" xr3:uid="{157A6765-6BEB-45C8-B059-14466701E200}" name="Imprint" dataDxfId="30"/>
+    <tableColumn id="3" xr3:uid="{C2D0AE15-8EB6-42FA-9756-6359A70C39F2}" name="Print ISSN" dataDxfId="29"/>
+    <tableColumn id="4" xr3:uid="{C1A14781-2EC2-4655-8B99-34C639B681F7}" name="Electronic ISSN" dataDxfId="28"/>
+    <tableColumn id="5" xr3:uid="{6A1CDB50-05D6-4137-BED6-66AEA762C1D8}" name="Journal URL" dataDxfId="27"/>
+    <tableColumn id="6" xr3:uid="{142F869A-41EF-4110-B212-DCDFE3A91B4D}" name="Publishing Model" dataDxfId="26"/>
+    <tableColumn id="7" xr3:uid="{883DC121-F62A-4717-ABC9-50C24089DAAE}" name="License Options" dataDxfId="25"/>
+    <tableColumn id="8" xr3:uid="{79ADE6AD-15D5-4E9E-ADB0-716C42F18B23}" name="Subject Areas" dataDxfId="24"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{50DE42A8-741C-4C2A-82B7-4C9C79D7B512}" name="Table14" displayName="Table14" ref="A4:J23" totalsRowShown="0" headerRowDxfId="25" dataDxfId="23" headerRowBorderDxfId="24" tableBorderDxfId="22" totalsRowBorderDxfId="21">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{50DE42A8-741C-4C2A-82B7-4C9C79D7B512}" name="Table14" displayName="Table14" ref="A4:J23" totalsRowShown="0" headerRowDxfId="23" dataDxfId="21" headerRowBorderDxfId="22" tableBorderDxfId="20" totalsRowBorderDxfId="19">
   <autoFilter ref="A4:J23" xr:uid="{50DE42A8-741C-4C2A-82B7-4C9C79D7B512}"/>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{1B9A1423-FE7E-41D7-B053-6BF091F459D2}" name="Journal Title" dataDxfId="20"/>
-    <tableColumn id="2" xr3:uid="{B625EB42-AF86-4F71-BC2F-65D99997CD50}" name="Imprint" dataDxfId="19"/>
-    <tableColumn id="3" xr3:uid="{559DDF72-C949-47E4-8DA4-297063A6725C}" name="Print ISSN" dataDxfId="18"/>
-    <tableColumn id="4" xr3:uid="{2C5C0518-FAE9-4E34-9C5C-031EDE4262BA}" name="Electronic ISSN" dataDxfId="17"/>
-    <tableColumn id="5" xr3:uid="{D5474278-5905-4A79-9DFE-DE4AB9980E12}" name="Journal URL" dataDxfId="16"/>
-    <tableColumn id="6" xr3:uid="{3D861C40-F9D7-4168-ACD1-389CE9995730}" name="Publishing Model" dataDxfId="15"/>
-    <tableColumn id="7" xr3:uid="{156C7878-43A4-40BA-84D1-0BD24E590EEE}" name="License Options" dataDxfId="14"/>
-    <tableColumn id="8" xr3:uid="{4C684C0B-6FA6-4E1F-BC47-B228FA209770}" name="Subject Areas" dataDxfId="13"/>
-    <tableColumn id="9" xr3:uid="{96CDE76D-4B76-48A4-98FB-70E2CCC4CFC8}" name="Change Type (See Terms)" dataDxfId="12"/>
-    <tableColumn id="10" xr3:uid="{43B192BA-2299-4882-A245-9C663CF7CF9B}" name="Change Note" dataDxfId="11"/>
+    <tableColumn id="1" xr3:uid="{1B9A1423-FE7E-41D7-B053-6BF091F459D2}" name="Journal Title" dataDxfId="18"/>
+    <tableColumn id="2" xr3:uid="{B625EB42-AF86-4F71-BC2F-65D99997CD50}" name="Imprint" dataDxfId="17"/>
+    <tableColumn id="3" xr3:uid="{559DDF72-C949-47E4-8DA4-297063A6725C}" name="Print ISSN" dataDxfId="16"/>
+    <tableColumn id="4" xr3:uid="{2C5C0518-FAE9-4E34-9C5C-031EDE4262BA}" name="Electronic ISSN" dataDxfId="15"/>
+    <tableColumn id="5" xr3:uid="{D5474278-5905-4A79-9DFE-DE4AB9980E12}" name="Journal URL" dataDxfId="14"/>
+    <tableColumn id="6" xr3:uid="{3D861C40-F9D7-4168-ACD1-389CE9995730}" name="Publishing Model" dataDxfId="13"/>
+    <tableColumn id="7" xr3:uid="{156C7878-43A4-40BA-84D1-0BD24E590EEE}" name="License Options" dataDxfId="12"/>
+    <tableColumn id="8" xr3:uid="{4C684C0B-6FA6-4E1F-BC47-B228FA209770}" name="Subject Areas" dataDxfId="11"/>
+    <tableColumn id="9" xr3:uid="{96CDE76D-4B76-48A4-98FB-70E2CCC4CFC8}" name="Change Type (See Terms)" dataDxfId="10"/>
+    <tableColumn id="10" xr3:uid="{43B192BA-2299-4882-A245-9C663CF7CF9B}" name="Change Note" dataDxfId="9"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{98A0D124-AED4-4DBE-8354-EE3315983F60}" name="Table25" displayName="Table25" ref="A1:B11" totalsRowShown="0" headerRowDxfId="10" dataDxfId="8" headerRowBorderDxfId="9" tableBorderDxfId="7" totalsRowBorderDxfId="6">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{98A0D124-AED4-4DBE-8354-EE3315983F60}" name="Table25" displayName="Table25" ref="A1:B11" totalsRowShown="0" headerRowDxfId="8" dataDxfId="6" headerRowBorderDxfId="7" tableBorderDxfId="5" totalsRowBorderDxfId="4">
   <autoFilter ref="A1:B11" xr:uid="{98A0D124-AED4-4DBE-8354-EE3315983F60}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B11">
     <sortCondition ref="A1:A11"/>
   </sortState>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{E088FFDE-8F3A-4B84-9B24-F82FF70FAEA5}" name="Term" dataDxfId="5"/>
-    <tableColumn id="2" xr3:uid="{3BB7484B-180C-438A-8248-E8FEA43CCABB}" name="Description" dataDxfId="4"/>
+    <tableColumn id="1" xr3:uid="{E088FFDE-8F3A-4B84-9B24-F82FF70FAEA5}" name="Term" dataDxfId="3"/>
+    <tableColumn id="2" xr3:uid="{3BB7484B-180C-438A-8248-E8FEA43CCABB}" name="Description" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2265,10 +2290,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D4A9487-D5B7-4CE1-99CD-1488FAF55674}">
-  <dimension ref="A1:K40"/>
+  <dimension ref="A1:K42"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="14.26953125" style="12" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="37.6328125" style="12" customWidth="1"/>
     <col min="2" max="2" width="9.1796875" style="12" customWidth="1"/>
     <col min="3" max="3" width="11.36328125" style="12" customWidth="1"/>
     <col min="4" max="4" width="16" style="12" customWidth="1"/>
@@ -2306,976 +2331,1024 @@
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A2" s="29" t="s">
+      <c r="A2" s="23" t="s">
+        <v>33</v>
+      </c>
+      <c r="B2" s="23" t="s">
+        <v>33</v>
+      </c>
+      <c r="C2"/>
+      <c r="D2" s="23" t="s">
+        <v>72</v>
+      </c>
+      <c r="E2" s="25" t="s">
+        <v>125</v>
+      </c>
+      <c r="F2" s="29" t="s">
+        <v>31</v>
+      </c>
+      <c r="G2" s="24" t="s">
+        <v>124</v>
+      </c>
+      <c r="H2" s="23" t="s">
+        <v>111</v>
+      </c>
+      <c r="J2"/>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A3" s="23" t="s">
+        <v>34</v>
+      </c>
+      <c r="B3" s="23" t="s">
+        <v>33</v>
+      </c>
+      <c r="C3"/>
+      <c r="D3" s="23" t="s">
+        <v>73</v>
+      </c>
+      <c r="E3" s="25" t="s">
+        <v>126</v>
+      </c>
+      <c r="F3" s="29" t="s">
+        <v>31</v>
+      </c>
+      <c r="G3" s="24" t="s">
+        <v>124</v>
+      </c>
+      <c r="H3" s="23" t="s">
+        <v>112</v>
+      </c>
+      <c r="J3"/>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A4" s="23" t="s">
+        <v>35</v>
+      </c>
+      <c r="B4" s="23" t="s">
+        <v>33</v>
+      </c>
+      <c r="C4"/>
+      <c r="D4" s="23" t="s">
+        <v>74</v>
+      </c>
+      <c r="E4" s="25" t="s">
+        <v>127</v>
+      </c>
+      <c r="F4" s="29" t="s">
+        <v>31</v>
+      </c>
+      <c r="G4" s="24" t="s">
+        <v>124</v>
+      </c>
+      <c r="H4" s="23" t="s">
+        <v>113</v>
+      </c>
+      <c r="J4"/>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A5" s="23" t="s">
+        <v>36</v>
+      </c>
+      <c r="B5" s="23" t="s">
+        <v>33</v>
+      </c>
+      <c r="C5"/>
+      <c r="D5" s="23" t="s">
+        <v>75</v>
+      </c>
+      <c r="E5" s="25" t="s">
+        <v>128</v>
+      </c>
+      <c r="F5" s="29" t="s">
+        <v>31</v>
+      </c>
+      <c r="G5" s="24" t="s">
+        <v>124</v>
+      </c>
+      <c r="H5" s="23" t="s">
+        <v>114</v>
+      </c>
+      <c r="J5"/>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A6" s="23" t="s">
+        <v>37</v>
+      </c>
+      <c r="B6" s="23" t="s">
+        <v>33</v>
+      </c>
+      <c r="C6"/>
+      <c r="D6" s="23" t="s">
+        <v>76</v>
+      </c>
+      <c r="E6" s="25" t="s">
+        <v>129</v>
+      </c>
+      <c r="F6" s="29" t="s">
+        <v>31</v>
+      </c>
+      <c r="G6" s="24" t="s">
+        <v>124</v>
+      </c>
+      <c r="H6" s="23" t="s">
+        <v>112</v>
+      </c>
+      <c r="J6"/>
+      <c r="K6" s="13"/>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A7" s="23" t="s">
+        <v>38</v>
+      </c>
+      <c r="B7" s="23" t="s">
+        <v>33</v>
+      </c>
+      <c r="C7"/>
+      <c r="D7" s="23" t="s">
+        <v>77</v>
+      </c>
+      <c r="E7" s="25" t="s">
+        <v>130</v>
+      </c>
+      <c r="F7" s="29" t="s">
+        <v>31</v>
+      </c>
+      <c r="G7" s="24" t="s">
+        <v>124</v>
+      </c>
+      <c r="H7" s="23" t="s">
+        <v>112</v>
+      </c>
+      <c r="J7"/>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A8" s="23" t="s">
+        <v>39</v>
+      </c>
+      <c r="B8" s="23" t="s">
+        <v>33</v>
+      </c>
+      <c r="C8"/>
+      <c r="D8" s="23" t="s">
+        <v>78</v>
+      </c>
+      <c r="E8" s="25" t="s">
+        <v>131</v>
+      </c>
+      <c r="F8" s="29" t="s">
+        <v>31</v>
+      </c>
+      <c r="G8" s="24" t="s">
+        <v>124</v>
+      </c>
+      <c r="H8" s="23" t="s">
+        <v>112</v>
+      </c>
+      <c r="J8"/>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A9" s="23" t="s">
+        <v>40</v>
+      </c>
+      <c r="B9" s="23" t="s">
+        <v>33</v>
+      </c>
+      <c r="C9"/>
+      <c r="D9" s="23" t="s">
+        <v>79</v>
+      </c>
+      <c r="E9" s="25" t="s">
+        <v>132</v>
+      </c>
+      <c r="F9" s="29" t="s">
+        <v>31</v>
+      </c>
+      <c r="G9" s="24" t="s">
+        <v>124</v>
+      </c>
+      <c r="H9" s="23" t="s">
+        <v>115</v>
+      </c>
+      <c r="J9"/>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A10" s="23" t="s">
+        <v>41</v>
+      </c>
+      <c r="B10" s="23" t="s">
+        <v>33</v>
+      </c>
+      <c r="C10"/>
+      <c r="D10" s="23" t="s">
+        <v>80</v>
+      </c>
+      <c r="E10" s="25" t="s">
+        <v>133</v>
+      </c>
+      <c r="F10" s="29" t="s">
+        <v>31</v>
+      </c>
+      <c r="G10" s="24" t="s">
+        <v>124</v>
+      </c>
+      <c r="H10" s="23" t="s">
+        <v>112</v>
+      </c>
+      <c r="J10"/>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A11" s="23" t="s">
         <v>42</v>
       </c>
-      <c r="B2" s="29" t="s">
-        <v>42</v>
-      </c>
-      <c r="C2"/>
-      <c r="D2" s="29" t="s">
+      <c r="B11" s="23" t="s">
+        <v>33</v>
+      </c>
+      <c r="C11"/>
+      <c r="D11" s="23" t="s">
         <v>81</v>
       </c>
-      <c r="E2" s="31" t="s">
+      <c r="E11" s="25" t="s">
+        <v>134</v>
+      </c>
+      <c r="F11" s="29" t="s">
+        <v>31</v>
+      </c>
+      <c r="G11" s="24" t="s">
+        <v>124</v>
+      </c>
+      <c r="H11" s="23" t="s">
+        <v>115</v>
+      </c>
+      <c r="J11"/>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A12" s="23" t="s">
+        <v>43</v>
+      </c>
+      <c r="B12" s="23" t="s">
+        <v>33</v>
+      </c>
+      <c r="C12"/>
+      <c r="D12" s="23" t="s">
+        <v>82</v>
+      </c>
+      <c r="E12" s="25" t="s">
         <v>135</v>
       </c>
-      <c r="F2" s="29" t="s">
-        <v>134</v>
-      </c>
-      <c r="G2" s="30" t="s">
-        <v>133</v>
-      </c>
-      <c r="H2" s="29" t="s">
+      <c r="F12" s="29" t="s">
+        <v>31</v>
+      </c>
+      <c r="G12" s="24" t="s">
+        <v>124</v>
+      </c>
+      <c r="H12" s="23" t="s">
+        <v>115</v>
+      </c>
+      <c r="J12"/>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A13" s="23" t="s">
+        <v>44</v>
+      </c>
+      <c r="B13" s="23" t="s">
+        <v>33</v>
+      </c>
+      <c r="C13"/>
+      <c r="D13" s="23" t="s">
+        <v>83</v>
+      </c>
+      <c r="E13" s="25" t="s">
+        <v>136</v>
+      </c>
+      <c r="F13" s="29" t="s">
+        <v>31</v>
+      </c>
+      <c r="G13" s="24" t="s">
+        <v>124</v>
+      </c>
+      <c r="H13" s="23" t="s">
+        <v>115</v>
+      </c>
+      <c r="J13"/>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A14" s="23" t="s">
+        <v>45</v>
+      </c>
+      <c r="B14" s="23" t="s">
+        <v>33</v>
+      </c>
+      <c r="C14"/>
+      <c r="D14" s="23" t="s">
+        <v>84</v>
+      </c>
+      <c r="E14" s="25" t="s">
+        <v>137</v>
+      </c>
+      <c r="F14" s="29" t="s">
+        <v>31</v>
+      </c>
+      <c r="G14" s="24" t="s">
+        <v>124</v>
+      </c>
+      <c r="H14" s="23" t="s">
+        <v>116</v>
+      </c>
+      <c r="J14"/>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A15" s="23" t="s">
+        <v>46</v>
+      </c>
+      <c r="B15" s="23" t="s">
+        <v>33</v>
+      </c>
+      <c r="C15"/>
+      <c r="D15" s="23" t="s">
+        <v>85</v>
+      </c>
+      <c r="E15" s="25" t="s">
+        <v>138</v>
+      </c>
+      <c r="F15" s="29" t="s">
+        <v>31</v>
+      </c>
+      <c r="G15" s="24" t="s">
+        <v>124</v>
+      </c>
+      <c r="H15" s="23" t="s">
+        <v>117</v>
+      </c>
+      <c r="J15"/>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A16" s="23" t="s">
+        <v>47</v>
+      </c>
+      <c r="B16" s="23" t="s">
+        <v>33</v>
+      </c>
+      <c r="C16"/>
+      <c r="D16" s="23" t="s">
+        <v>86</v>
+      </c>
+      <c r="E16" s="25" t="s">
+        <v>139</v>
+      </c>
+      <c r="F16" s="29" t="s">
+        <v>31</v>
+      </c>
+      <c r="G16" s="24" t="s">
+        <v>124</v>
+      </c>
+      <c r="H16" s="23" t="s">
+        <v>118</v>
+      </c>
+      <c r="J16"/>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A17" s="23" t="s">
+        <v>48</v>
+      </c>
+      <c r="B17" s="23" t="s">
+        <v>33</v>
+      </c>
+      <c r="C17"/>
+      <c r="D17" s="23" t="s">
+        <v>87</v>
+      </c>
+      <c r="E17" s="25" t="s">
+        <v>140</v>
+      </c>
+      <c r="F17" s="29" t="s">
+        <v>31</v>
+      </c>
+      <c r="G17" s="24" t="s">
+        <v>124</v>
+      </c>
+      <c r="H17" s="23" t="s">
+        <v>112</v>
+      </c>
+      <c r="J17"/>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A18" s="30" t="s">
+        <v>49</v>
+      </c>
+      <c r="B18" s="30" t="s">
+        <v>33</v>
+      </c>
+      <c r="C18" s="27"/>
+      <c r="D18" s="30" t="s">
+        <v>88</v>
+      </c>
+      <c r="E18" s="31" t="s">
+        <v>141</v>
+      </c>
+      <c r="F18" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="G18" s="33" t="s">
+        <v>124</v>
+      </c>
+      <c r="H18" s="30" t="s">
+        <v>119</v>
+      </c>
+      <c r="J18"/>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A19" s="30" t="s">
+        <v>50</v>
+      </c>
+      <c r="B19" s="30" t="s">
+        <v>33</v>
+      </c>
+      <c r="C19" s="27"/>
+      <c r="D19" s="30" t="s">
+        <v>89</v>
+      </c>
+      <c r="E19" s="31" t="s">
+        <v>142</v>
+      </c>
+      <c r="F19" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="G19" s="33" t="s">
+        <v>124</v>
+      </c>
+      <c r="H19" s="30" t="s">
         <v>120</v>
       </c>
-      <c r="J2"/>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A3" s="29" t="s">
-        <v>43</v>
-      </c>
-      <c r="B3" s="29" t="s">
-        <v>42</v>
-      </c>
-      <c r="C3"/>
-      <c r="D3" s="29" t="s">
-        <v>82</v>
-      </c>
-      <c r="E3" s="31" t="s">
-        <v>136</v>
-      </c>
-      <c r="F3" s="29" t="s">
-        <v>134</v>
-      </c>
-      <c r="G3" s="30" t="s">
-        <v>133</v>
-      </c>
-      <c r="H3" s="29" t="s">
+      <c r="J19"/>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A20" s="30" t="s">
+        <v>51</v>
+      </c>
+      <c r="B20" s="30" t="s">
+        <v>33</v>
+      </c>
+      <c r="C20" s="27"/>
+      <c r="D20" s="30" t="s">
+        <v>90</v>
+      </c>
+      <c r="E20" s="31" t="s">
+        <v>143</v>
+      </c>
+      <c r="F20" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="G20" s="33" t="s">
+        <v>124</v>
+      </c>
+      <c r="H20" s="30" t="s">
+        <v>111</v>
+      </c>
+      <c r="J20"/>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A21" s="30" t="s">
+        <v>52</v>
+      </c>
+      <c r="B21" s="30" t="s">
+        <v>33</v>
+      </c>
+      <c r="C21" s="27"/>
+      <c r="D21" s="30" t="s">
+        <v>91</v>
+      </c>
+      <c r="E21" s="31" t="s">
+        <v>144</v>
+      </c>
+      <c r="F21" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="G21" s="33" t="s">
+        <v>124</v>
+      </c>
+      <c r="H21" s="30" t="s">
+        <v>114</v>
+      </c>
+      <c r="J21"/>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A22" s="30" t="s">
+        <v>53</v>
+      </c>
+      <c r="B22" s="30" t="s">
+        <v>33</v>
+      </c>
+      <c r="C22" s="27"/>
+      <c r="D22" s="30" t="s">
+        <v>92</v>
+      </c>
+      <c r="E22" s="31" t="s">
+        <v>145</v>
+      </c>
+      <c r="F22" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="G22" s="33" t="s">
+        <v>124</v>
+      </c>
+      <c r="H22" s="30" t="s">
         <v>121</v>
       </c>
-      <c r="J3"/>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A4" s="29" t="s">
-        <v>44</v>
-      </c>
-      <c r="B4" s="29" t="s">
-        <v>42</v>
-      </c>
-      <c r="C4"/>
-      <c r="D4" s="29" t="s">
-        <v>83</v>
-      </c>
-      <c r="E4" s="31" t="s">
-        <v>137</v>
-      </c>
-      <c r="F4" s="29" t="s">
-        <v>134</v>
-      </c>
-      <c r="G4" s="30" t="s">
-        <v>133</v>
-      </c>
-      <c r="H4" s="29" t="s">
+      <c r="J22"/>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A23" s="30" t="s">
+        <v>54</v>
+      </c>
+      <c r="B23" s="30" t="s">
+        <v>33</v>
+      </c>
+      <c r="C23" s="27"/>
+      <c r="D23" s="30" t="s">
+        <v>93</v>
+      </c>
+      <c r="E23" s="31" t="s">
+        <v>146</v>
+      </c>
+      <c r="F23" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="G23" s="33" t="s">
+        <v>124</v>
+      </c>
+      <c r="H23" s="30" t="s">
+        <v>112</v>
+      </c>
+      <c r="J23"/>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A24" s="30" t="s">
+        <v>55</v>
+      </c>
+      <c r="B24" s="30" t="s">
+        <v>33</v>
+      </c>
+      <c r="C24" s="27"/>
+      <c r="D24" s="30" t="s">
+        <v>94</v>
+      </c>
+      <c r="E24" s="31" t="s">
+        <v>147</v>
+      </c>
+      <c r="F24" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="G24" s="33" t="s">
+        <v>124</v>
+      </c>
+      <c r="H24" s="30" t="s">
+        <v>114</v>
+      </c>
+      <c r="J24"/>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A25" s="30" t="s">
+        <v>56</v>
+      </c>
+      <c r="B25" s="30" t="s">
+        <v>33</v>
+      </c>
+      <c r="C25" s="27"/>
+      <c r="D25" s="30" t="s">
+        <v>95</v>
+      </c>
+      <c r="E25" s="31" t="s">
+        <v>148</v>
+      </c>
+      <c r="F25" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="G25" s="33" t="s">
+        <v>124</v>
+      </c>
+      <c r="H25" s="30" t="s">
+        <v>119</v>
+      </c>
+      <c r="J25"/>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A26" s="30" t="s">
+        <v>57</v>
+      </c>
+      <c r="B26" s="30" t="s">
+        <v>33</v>
+      </c>
+      <c r="C26" s="27"/>
+      <c r="D26" s="30" t="s">
+        <v>96</v>
+      </c>
+      <c r="E26" s="31" t="s">
+        <v>149</v>
+      </c>
+      <c r="F26" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="G26" s="33" t="s">
+        <v>124</v>
+      </c>
+      <c r="H26" s="30" t="s">
         <v>122</v>
       </c>
-      <c r="J4"/>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A5" s="29" t="s">
-        <v>45</v>
-      </c>
-      <c r="B5" s="29" t="s">
-        <v>42</v>
-      </c>
-      <c r="C5"/>
-      <c r="D5" s="29" t="s">
-        <v>84</v>
-      </c>
-      <c r="E5" s="31" t="s">
-        <v>138</v>
-      </c>
-      <c r="F5" s="29" t="s">
-        <v>134</v>
-      </c>
-      <c r="G5" s="30" t="s">
-        <v>133</v>
-      </c>
-      <c r="H5" s="29" t="s">
+      <c r="J26"/>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A27" s="30" t="s">
+        <v>58</v>
+      </c>
+      <c r="B27" s="30" t="s">
+        <v>33</v>
+      </c>
+      <c r="C27" s="27"/>
+      <c r="D27" s="30" t="s">
+        <v>97</v>
+      </c>
+      <c r="E27" s="31" t="s">
+        <v>150</v>
+      </c>
+      <c r="F27" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="G27" s="33" t="s">
+        <v>124</v>
+      </c>
+      <c r="H27" s="30" t="s">
+        <v>114</v>
+      </c>
+      <c r="J27"/>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A28" s="30" t="s">
+        <v>59</v>
+      </c>
+      <c r="B28" s="30" t="s">
+        <v>33</v>
+      </c>
+      <c r="C28" s="27"/>
+      <c r="D28" s="30" t="s">
+        <v>98</v>
+      </c>
+      <c r="E28" s="31" t="s">
+        <v>151</v>
+      </c>
+      <c r="F28" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="G28" s="33" t="s">
+        <v>124</v>
+      </c>
+      <c r="H28" s="30" t="s">
         <v>123</v>
       </c>
-      <c r="J5"/>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A6" s="29" t="s">
-        <v>46</v>
-      </c>
-      <c r="B6" s="29" t="s">
-        <v>42</v>
-      </c>
-      <c r="C6"/>
-      <c r="D6" s="29" t="s">
-        <v>85</v>
-      </c>
-      <c r="E6" s="31" t="s">
-        <v>139</v>
-      </c>
-      <c r="F6" s="29" t="s">
-        <v>134</v>
-      </c>
-      <c r="G6" s="30" t="s">
-        <v>133</v>
-      </c>
-      <c r="H6" s="29" t="s">
-        <v>121</v>
-      </c>
-      <c r="J6"/>
-      <c r="K6" s="14"/>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A7" s="29" t="s">
-        <v>47</v>
-      </c>
-      <c r="B7" s="29" t="s">
-        <v>42</v>
-      </c>
-      <c r="C7"/>
-      <c r="D7" s="29" t="s">
-        <v>86</v>
-      </c>
-      <c r="E7" s="31" t="s">
-        <v>140</v>
-      </c>
-      <c r="F7" s="29" t="s">
-        <v>134</v>
-      </c>
-      <c r="G7" s="30" t="s">
-        <v>133</v>
-      </c>
-      <c r="H7" s="29" t="s">
-        <v>121</v>
-      </c>
-      <c r="J7"/>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A8" s="29" t="s">
-        <v>48</v>
-      </c>
-      <c r="B8" s="29" t="s">
-        <v>42</v>
-      </c>
-      <c r="C8"/>
-      <c r="D8" s="29" t="s">
-        <v>87</v>
-      </c>
-      <c r="E8" s="31" t="s">
-        <v>141</v>
-      </c>
-      <c r="F8" s="29" t="s">
-        <v>134</v>
-      </c>
-      <c r="G8" s="30" t="s">
-        <v>133</v>
-      </c>
-      <c r="H8" s="29" t="s">
-        <v>121</v>
-      </c>
-      <c r="J8"/>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A9" s="29" t="s">
-        <v>49</v>
-      </c>
-      <c r="B9" s="29" t="s">
-        <v>42</v>
-      </c>
-      <c r="C9"/>
-      <c r="D9" s="29" t="s">
-        <v>88</v>
-      </c>
-      <c r="E9" s="31" t="s">
-        <v>142</v>
-      </c>
-      <c r="F9" s="29" t="s">
-        <v>134</v>
-      </c>
-      <c r="G9" s="30" t="s">
-        <v>133</v>
-      </c>
-      <c r="H9" s="29" t="s">
-        <v>124</v>
-      </c>
-      <c r="J9"/>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A10" s="29" t="s">
-        <v>50</v>
-      </c>
-      <c r="B10" s="29" t="s">
-        <v>42</v>
-      </c>
-      <c r="C10"/>
-      <c r="D10" s="29" t="s">
-        <v>89</v>
-      </c>
-      <c r="E10" s="31" t="s">
-        <v>143</v>
-      </c>
-      <c r="F10" s="29" t="s">
-        <v>134</v>
-      </c>
-      <c r="G10" s="30" t="s">
-        <v>133</v>
-      </c>
-      <c r="H10" s="29" t="s">
-        <v>121</v>
-      </c>
-      <c r="J10"/>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A11" s="29" t="s">
-        <v>51</v>
-      </c>
-      <c r="B11" s="29" t="s">
-        <v>42</v>
-      </c>
-      <c r="C11"/>
-      <c r="D11" s="29" t="s">
-        <v>90</v>
-      </c>
-      <c r="E11" s="31" t="s">
-        <v>144</v>
-      </c>
-      <c r="F11" s="29" t="s">
-        <v>134</v>
-      </c>
-      <c r="G11" s="30" t="s">
-        <v>133</v>
-      </c>
-      <c r="H11" s="29" t="s">
-        <v>124</v>
-      </c>
-      <c r="J11"/>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A12" s="29" t="s">
-        <v>52</v>
-      </c>
-      <c r="B12" s="29" t="s">
-        <v>42</v>
-      </c>
-      <c r="C12"/>
-      <c r="D12" s="29" t="s">
-        <v>91</v>
-      </c>
-      <c r="E12" s="31" t="s">
-        <v>145</v>
-      </c>
-      <c r="F12" s="29" t="s">
-        <v>134</v>
-      </c>
-      <c r="G12" s="30" t="s">
-        <v>133</v>
-      </c>
-      <c r="H12" s="29" t="s">
-        <v>124</v>
-      </c>
-      <c r="J12"/>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A13" s="29" t="s">
-        <v>53</v>
-      </c>
-      <c r="B13" s="29" t="s">
-        <v>42</v>
-      </c>
-      <c r="C13"/>
-      <c r="D13" s="29" t="s">
-        <v>92</v>
-      </c>
-      <c r="E13" s="31" t="s">
-        <v>146</v>
-      </c>
-      <c r="F13" s="29" t="s">
-        <v>134</v>
-      </c>
-      <c r="G13" s="30" t="s">
-        <v>133</v>
-      </c>
-      <c r="H13" s="29" t="s">
-        <v>124</v>
-      </c>
-      <c r="J13"/>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A14" s="29" t="s">
-        <v>54</v>
-      </c>
-      <c r="B14" s="29" t="s">
-        <v>42</v>
-      </c>
-      <c r="C14"/>
-      <c r="D14" s="29" t="s">
-        <v>93</v>
-      </c>
-      <c r="E14" s="31" t="s">
-        <v>147</v>
-      </c>
-      <c r="F14" s="29" t="s">
-        <v>134</v>
-      </c>
-      <c r="G14" s="30" t="s">
-        <v>133</v>
-      </c>
-      <c r="H14" s="29" t="s">
-        <v>125</v>
-      </c>
-      <c r="J14"/>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A15" s="29" t="s">
-        <v>55</v>
-      </c>
-      <c r="B15" s="29" t="s">
-        <v>42</v>
-      </c>
-      <c r="C15"/>
-      <c r="D15" s="29" t="s">
-        <v>94</v>
-      </c>
-      <c r="E15" s="31" t="s">
-        <v>148</v>
-      </c>
-      <c r="F15" s="29" t="s">
-        <v>134</v>
-      </c>
-      <c r="G15" s="30" t="s">
-        <v>133</v>
-      </c>
-      <c r="H15" s="29" t="s">
-        <v>126</v>
-      </c>
-      <c r="J15"/>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A16" s="29" t="s">
-        <v>56</v>
-      </c>
-      <c r="B16" s="29" t="s">
-        <v>42</v>
-      </c>
-      <c r="C16"/>
-      <c r="D16" s="29" t="s">
-        <v>95</v>
-      </c>
-      <c r="E16" s="31" t="s">
-        <v>149</v>
-      </c>
-      <c r="F16" s="29" t="s">
-        <v>134</v>
-      </c>
-      <c r="G16" s="30" t="s">
-        <v>133</v>
-      </c>
-      <c r="H16" s="29" t="s">
-        <v>127</v>
-      </c>
-      <c r="J16"/>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A17" s="29" t="s">
-        <v>57</v>
-      </c>
-      <c r="B17" s="29" t="s">
-        <v>42</v>
-      </c>
-      <c r="C17"/>
-      <c r="D17" s="29" t="s">
-        <v>96</v>
-      </c>
-      <c r="E17" s="31" t="s">
-        <v>150</v>
-      </c>
-      <c r="F17" s="29" t="s">
-        <v>134</v>
-      </c>
-      <c r="G17" s="30" t="s">
-        <v>133</v>
-      </c>
-      <c r="H17" s="29" t="s">
-        <v>121</v>
-      </c>
-      <c r="J17"/>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A18" s="29" t="s">
-        <v>58</v>
-      </c>
-      <c r="B18" s="29" t="s">
-        <v>42</v>
-      </c>
-      <c r="C18"/>
-      <c r="D18" s="29" t="s">
-        <v>97</v>
-      </c>
-      <c r="E18" s="31" t="s">
-        <v>151</v>
-      </c>
-      <c r="F18" s="29" t="s">
-        <v>134</v>
-      </c>
-      <c r="G18" s="30" t="s">
-        <v>133</v>
-      </c>
-      <c r="H18" s="29" t="s">
-        <v>128</v>
-      </c>
-      <c r="J18"/>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A19" s="29" t="s">
-        <v>59</v>
-      </c>
-      <c r="B19" s="29" t="s">
-        <v>42</v>
-      </c>
-      <c r="C19"/>
-      <c r="D19" s="29" t="s">
-        <v>98</v>
-      </c>
-      <c r="E19" s="31" t="s">
+      <c r="J28"/>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A29" s="30" t="s">
+        <v>60</v>
+      </c>
+      <c r="B29" s="30" t="s">
+        <v>33</v>
+      </c>
+      <c r="C29" s="27"/>
+      <c r="D29" s="30" t="s">
+        <v>99</v>
+      </c>
+      <c r="E29" s="31" t="s">
         <v>152</v>
       </c>
-      <c r="F19" s="29" t="s">
-        <v>134</v>
-      </c>
-      <c r="G19" s="30" t="s">
-        <v>133</v>
-      </c>
-      <c r="H19" s="29" t="s">
-        <v>129</v>
-      </c>
-      <c r="J19"/>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A20" s="29" t="s">
-        <v>60</v>
-      </c>
-      <c r="B20" s="29" t="s">
-        <v>42</v>
-      </c>
-      <c r="C20"/>
-      <c r="D20" s="29" t="s">
-        <v>99</v>
-      </c>
-      <c r="E20" s="31" t="s">
+      <c r="F29" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="G29" s="33" t="s">
+        <v>124</v>
+      </c>
+      <c r="H29" s="30" t="s">
+        <v>112</v>
+      </c>
+      <c r="J29"/>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A30" s="30" t="s">
+        <v>61</v>
+      </c>
+      <c r="B30" s="30" t="s">
+        <v>33</v>
+      </c>
+      <c r="C30" s="27"/>
+      <c r="D30" s="30" t="s">
+        <v>100</v>
+      </c>
+      <c r="E30" s="31" t="s">
         <v>153</v>
       </c>
-      <c r="F20" s="29" t="s">
-        <v>134</v>
-      </c>
-      <c r="G20" s="30" t="s">
-        <v>133</v>
-      </c>
-      <c r="H20" s="29" t="s">
-        <v>120</v>
-      </c>
-      <c r="J20"/>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A21" s="29" t="s">
-        <v>61</v>
-      </c>
-      <c r="B21" s="29" t="s">
-        <v>42</v>
-      </c>
-      <c r="C21"/>
-      <c r="D21" s="29" t="s">
-        <v>100</v>
-      </c>
-      <c r="E21" s="31" t="s">
+      <c r="F30" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="G30" s="33" t="s">
+        <v>124</v>
+      </c>
+      <c r="H30" s="30" t="s">
+        <v>112</v>
+      </c>
+      <c r="J30"/>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A31" s="30" t="s">
+        <v>62</v>
+      </c>
+      <c r="B31" s="30" t="s">
+        <v>33</v>
+      </c>
+      <c r="C31" s="27"/>
+      <c r="D31" s="30" t="s">
+        <v>101</v>
+      </c>
+      <c r="E31" s="31" t="s">
+        <v>155</v>
+      </c>
+      <c r="F31" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="G31" s="33" t="s">
+        <v>124</v>
+      </c>
+      <c r="H31" s="30" t="s">
+        <v>112</v>
+      </c>
+      <c r="J31"/>
+    </row>
+    <row r="32" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A32" s="30" t="s">
+        <v>63</v>
+      </c>
+      <c r="B32" s="30" t="s">
+        <v>33</v>
+      </c>
+      <c r="C32" s="34"/>
+      <c r="D32" s="30" t="s">
+        <v>102</v>
+      </c>
+      <c r="E32" s="30" t="s">
         <v>154</v>
       </c>
-      <c r="F21" s="29" t="s">
-        <v>134</v>
-      </c>
-      <c r="G21" s="30" t="s">
-        <v>133</v>
-      </c>
-      <c r="H21" s="29" t="s">
-        <v>123</v>
-      </c>
-      <c r="J21"/>
-    </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A22" s="29" t="s">
-        <v>62</v>
-      </c>
-      <c r="B22" s="29" t="s">
-        <v>42</v>
-      </c>
-      <c r="C22"/>
-      <c r="D22" s="29" t="s">
-        <v>101</v>
-      </c>
-      <c r="E22" s="31" t="s">
-        <v>155</v>
-      </c>
-      <c r="F22" s="29" t="s">
-        <v>134</v>
-      </c>
-      <c r="G22" s="30" t="s">
-        <v>133</v>
-      </c>
-      <c r="H22" s="29" t="s">
-        <v>130</v>
-      </c>
-      <c r="J22"/>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A23" s="29" t="s">
-        <v>63</v>
-      </c>
-      <c r="B23" s="29" t="s">
-        <v>42</v>
-      </c>
-      <c r="C23"/>
-      <c r="D23" s="29" t="s">
-        <v>102</v>
-      </c>
-      <c r="E23" s="31" t="s">
+      <c r="F32" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="G32" s="33" t="s">
+        <v>124</v>
+      </c>
+      <c r="H32" s="30" t="s">
+        <v>122</v>
+      </c>
+      <c r="J32"/>
+    </row>
+    <row r="33" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A33" s="30" t="s">
+        <v>64</v>
+      </c>
+      <c r="B33" s="30" t="s">
+        <v>33</v>
+      </c>
+      <c r="C33" s="34"/>
+      <c r="D33" s="30" t="s">
+        <v>103</v>
+      </c>
+      <c r="E33" s="30" t="s">
         <v>156</v>
       </c>
-      <c r="F23" s="29" t="s">
-        <v>134</v>
-      </c>
-      <c r="G23" s="30" t="s">
-        <v>133</v>
-      </c>
-      <c r="H23" s="29" t="s">
-        <v>121</v>
-      </c>
-      <c r="J23"/>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A24" s="29" t="s">
-        <v>64</v>
-      </c>
-      <c r="B24" s="29" t="s">
-        <v>42</v>
-      </c>
-      <c r="C24"/>
-      <c r="D24" s="29" t="s">
-        <v>103</v>
-      </c>
-      <c r="E24" s="31" t="s">
+      <c r="F33" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="G33" s="33" t="s">
+        <v>124</v>
+      </c>
+      <c r="H33" s="30" t="s">
+        <v>114</v>
+      </c>
+      <c r="J33"/>
+    </row>
+    <row r="34" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A34" s="30" t="s">
+        <v>65</v>
+      </c>
+      <c r="B34" s="30" t="s">
+        <v>33</v>
+      </c>
+      <c r="C34" s="34"/>
+      <c r="D34" s="30" t="s">
+        <v>104</v>
+      </c>
+      <c r="E34" s="30" t="s">
         <v>157</v>
       </c>
-      <c r="F24" s="29" t="s">
-        <v>134</v>
-      </c>
-      <c r="G24" s="30" t="s">
-        <v>133</v>
-      </c>
-      <c r="H24" s="29" t="s">
-        <v>123</v>
-      </c>
-      <c r="J24"/>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A25" s="29" t="s">
-        <v>65</v>
-      </c>
-      <c r="B25" s="29" t="s">
-        <v>42</v>
-      </c>
-      <c r="C25"/>
-      <c r="D25" s="29" t="s">
-        <v>104</v>
-      </c>
-      <c r="E25" s="31" t="s">
+      <c r="F34" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="G34" s="33" t="s">
+        <v>124</v>
+      </c>
+      <c r="H34" s="30" t="s">
+        <v>113</v>
+      </c>
+      <c r="J34"/>
+    </row>
+    <row r="35" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A35" s="30" t="s">
+        <v>66</v>
+      </c>
+      <c r="B35" s="30" t="s">
+        <v>33</v>
+      </c>
+      <c r="C35" s="34"/>
+      <c r="D35" s="30" t="s">
+        <v>105</v>
+      </c>
+      <c r="E35" s="30" t="s">
         <v>158</v>
       </c>
-      <c r="F25" s="29" t="s">
-        <v>134</v>
-      </c>
-      <c r="G25" s="30" t="s">
-        <v>133</v>
-      </c>
-      <c r="H25" s="29" t="s">
-        <v>128</v>
-      </c>
-      <c r="J25"/>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A26" s="29" t="s">
-        <v>66</v>
-      </c>
-      <c r="B26" s="29" t="s">
-        <v>42</v>
-      </c>
-      <c r="C26"/>
-      <c r="D26" s="29" t="s">
-        <v>105</v>
-      </c>
-      <c r="E26" s="31" t="s">
+      <c r="F35" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="G35" s="33" t="s">
+        <v>124</v>
+      </c>
+      <c r="H35" s="30" t="s">
+        <v>113</v>
+      </c>
+      <c r="J35"/>
+    </row>
+    <row r="36" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A36" s="30" t="s">
+        <v>67</v>
+      </c>
+      <c r="B36" s="30" t="s">
+        <v>33</v>
+      </c>
+      <c r="C36" s="34"/>
+      <c r="D36" s="30" t="s">
+        <v>106</v>
+      </c>
+      <c r="E36" s="30" t="s">
         <v>159</v>
       </c>
-      <c r="F26" s="29" t="s">
-        <v>134</v>
-      </c>
-      <c r="G26" s="30" t="s">
-        <v>133</v>
-      </c>
-      <c r="H26" s="29" t="s">
-        <v>131</v>
-      </c>
-      <c r="J26"/>
-    </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A27" s="29" t="s">
-        <v>67</v>
-      </c>
-      <c r="B27" s="29" t="s">
-        <v>42</v>
-      </c>
-      <c r="C27"/>
-      <c r="D27" s="29" t="s">
-        <v>106</v>
-      </c>
-      <c r="E27" s="31" t="s">
+      <c r="F36" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="G36" s="33" t="s">
+        <v>124</v>
+      </c>
+      <c r="H36" s="30" t="s">
+        <v>112</v>
+      </c>
+      <c r="J36"/>
+    </row>
+    <row r="37" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A37" s="30" t="s">
+        <v>68</v>
+      </c>
+      <c r="B37" s="30" t="s">
+        <v>33</v>
+      </c>
+      <c r="C37" s="34"/>
+      <c r="D37" s="30" t="s">
+        <v>107</v>
+      </c>
+      <c r="E37" s="30" t="s">
         <v>160</v>
       </c>
-      <c r="F27" s="29" t="s">
-        <v>134</v>
-      </c>
-      <c r="G27" s="30" t="s">
-        <v>133</v>
-      </c>
-      <c r="H27" s="29" t="s">
-        <v>123</v>
-      </c>
-      <c r="J27"/>
-    </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A28" s="29" t="s">
-        <v>68</v>
-      </c>
-      <c r="B28" s="29" t="s">
-        <v>42</v>
-      </c>
-      <c r="C28"/>
-      <c r="D28" s="29" t="s">
-        <v>107</v>
-      </c>
-      <c r="E28" s="31" t="s">
+      <c r="F37" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="G37" s="33" t="s">
+        <v>124</v>
+      </c>
+      <c r="H37" s="30" t="s">
+        <v>112</v>
+      </c>
+      <c r="J37"/>
+    </row>
+    <row r="38" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A38" s="30" t="s">
+        <v>69</v>
+      </c>
+      <c r="B38" s="30" t="s">
+        <v>33</v>
+      </c>
+      <c r="C38" s="34"/>
+      <c r="D38" s="30" t="s">
+        <v>108</v>
+      </c>
+      <c r="E38" s="30" t="s">
         <v>161</v>
       </c>
-      <c r="F28" s="29" t="s">
-        <v>134</v>
-      </c>
-      <c r="G28" s="30" t="s">
-        <v>133</v>
-      </c>
-      <c r="H28" s="29" t="s">
-        <v>132</v>
-      </c>
-      <c r="J28"/>
-    </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A29" s="29" t="s">
-        <v>69</v>
-      </c>
-      <c r="B29" s="29" t="s">
-        <v>42</v>
-      </c>
-      <c r="C29"/>
-      <c r="D29" s="29" t="s">
-        <v>108</v>
-      </c>
-      <c r="E29" s="31" t="s">
+      <c r="F38" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="G38" s="33" t="s">
+        <v>124</v>
+      </c>
+      <c r="H38" s="30" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A39" s="30" t="s">
+        <v>70</v>
+      </c>
+      <c r="B39" s="30" t="s">
+        <v>33</v>
+      </c>
+      <c r="C39" s="34"/>
+      <c r="D39" s="30" t="s">
+        <v>109</v>
+      </c>
+      <c r="E39" s="30" t="s">
         <v>162</v>
       </c>
-      <c r="F29" s="29" t="s">
-        <v>134</v>
-      </c>
-      <c r="G29" s="30" t="s">
-        <v>133</v>
-      </c>
-      <c r="H29" s="29" t="s">
-        <v>121</v>
-      </c>
-      <c r="J29"/>
-    </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A30" s="29" t="s">
-        <v>70</v>
-      </c>
-      <c r="B30" s="29" t="s">
-        <v>42</v>
-      </c>
-      <c r="C30"/>
-      <c r="D30" s="29" t="s">
-        <v>109</v>
-      </c>
-      <c r="E30" s="31" t="s">
+      <c r="F39" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="G39" s="33" t="s">
+        <v>124</v>
+      </c>
+      <c r="H39" s="30" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A40" s="30" t="s">
+        <v>71</v>
+      </c>
+      <c r="B40" s="30" t="s">
+        <v>33</v>
+      </c>
+      <c r="C40" s="34"/>
+      <c r="D40" s="30" t="s">
+        <v>110</v>
+      </c>
+      <c r="E40" s="30" t="s">
         <v>163</v>
       </c>
-      <c r="F30" s="29" t="s">
-        <v>134</v>
-      </c>
-      <c r="G30" s="30" t="s">
-        <v>133</v>
-      </c>
-      <c r="H30" s="29" t="s">
-        <v>121</v>
-      </c>
-      <c r="J30"/>
-    </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A31" s="29" t="s">
-        <v>71</v>
-      </c>
-      <c r="B31" s="29" t="s">
-        <v>42</v>
-      </c>
-      <c r="C31"/>
-      <c r="D31" s="29" t="s">
-        <v>110</v>
-      </c>
-      <c r="E31" s="31" t="s">
+      <c r="F40" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="G40" s="33" t="s">
+        <v>124</v>
+      </c>
+      <c r="H40" s="30" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A41" s="35" t="s">
+        <v>166</v>
+      </c>
+      <c r="B41" s="30" t="s">
+        <v>33</v>
+      </c>
+      <c r="C41" s="36"/>
+      <c r="D41" s="35" t="s">
         <v>165</v>
       </c>
-      <c r="F31" s="29" t="s">
-        <v>134</v>
-      </c>
-      <c r="G31" s="30" t="s">
-        <v>133</v>
-      </c>
-      <c r="H31" s="29" t="s">
-        <v>121</v>
-      </c>
-      <c r="J31"/>
-    </row>
-    <row r="32" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A32" s="29" t="s">
-        <v>72</v>
-      </c>
-      <c r="B32" s="29" t="s">
-        <v>42</v>
-      </c>
-      <c r="C32" s="13"/>
-      <c r="D32" s="29" t="s">
-        <v>111</v>
-      </c>
-      <c r="E32" s="29" t="s">
+      <c r="E41" s="28" t="s">
+        <v>171</v>
+      </c>
+      <c r="F41" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="G41" s="33" t="s">
+        <v>124</v>
+      </c>
+      <c r="H41" s="37" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10" ht="46.5" x14ac:dyDescent="0.35">
+      <c r="A42" s="35" t="s">
+        <v>167</v>
+      </c>
+      <c r="B42" s="30" t="s">
+        <v>33</v>
+      </c>
+      <c r="C42" s="36"/>
+      <c r="D42" s="37" t="s">
         <v>164</v>
       </c>
-      <c r="F32" s="29" t="s">
-        <v>134</v>
-      </c>
-      <c r="G32" s="30" t="s">
-        <v>133</v>
-      </c>
-      <c r="H32" s="29" t="s">
-        <v>131</v>
-      </c>
-      <c r="J32"/>
-    </row>
-    <row r="33" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A33" s="29" t="s">
-        <v>73</v>
-      </c>
-      <c r="B33" s="29" t="s">
-        <v>42</v>
-      </c>
-      <c r="C33" s="13"/>
-      <c r="D33" s="29" t="s">
-        <v>112</v>
-      </c>
-      <c r="E33" s="29" t="s">
-        <v>166</v>
-      </c>
-      <c r="F33" s="29" t="s">
-        <v>134</v>
-      </c>
-      <c r="G33" s="30" t="s">
-        <v>133</v>
-      </c>
-      <c r="H33" s="29" t="s">
-        <v>123</v>
-      </c>
-      <c r="J33"/>
-    </row>
-    <row r="34" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A34" s="29" t="s">
-        <v>74</v>
-      </c>
-      <c r="B34" s="29" t="s">
-        <v>42</v>
-      </c>
-      <c r="C34" s="13"/>
-      <c r="D34" s="29" t="s">
-        <v>113</v>
-      </c>
-      <c r="E34" s="29" t="s">
-        <v>167</v>
-      </c>
-      <c r="F34" s="29" t="s">
-        <v>134</v>
-      </c>
-      <c r="G34" s="30" t="s">
-        <v>133</v>
-      </c>
-      <c r="H34" s="29" t="s">
-        <v>122</v>
-      </c>
-      <c r="J34"/>
-    </row>
-    <row r="35" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A35" s="29" t="s">
-        <v>75</v>
-      </c>
-      <c r="B35" s="29" t="s">
-        <v>42</v>
-      </c>
-      <c r="C35" s="13"/>
-      <c r="D35" s="29" t="s">
-        <v>114</v>
-      </c>
-      <c r="E35" s="29" t="s">
-        <v>168</v>
-      </c>
-      <c r="F35" s="29" t="s">
-        <v>134</v>
-      </c>
-      <c r="G35" s="30" t="s">
-        <v>133</v>
-      </c>
-      <c r="H35" s="29" t="s">
-        <v>122</v>
-      </c>
-      <c r="J35"/>
-    </row>
-    <row r="36" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A36" s="29" t="s">
-        <v>76</v>
-      </c>
-      <c r="B36" s="29" t="s">
-        <v>42</v>
-      </c>
-      <c r="C36" s="13"/>
-      <c r="D36" s="29" t="s">
-        <v>115</v>
-      </c>
-      <c r="E36" s="29" t="s">
+      <c r="E42" s="36" t="s">
+        <v>170</v>
+      </c>
+      <c r="F42" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="G42" s="33" t="s">
+        <v>124</v>
+      </c>
+      <c r="H42" s="37" t="s">
         <v>169</v>
-      </c>
-      <c r="F36" s="29" t="s">
-        <v>134</v>
-      </c>
-      <c r="G36" s="30" t="s">
-        <v>133</v>
-      </c>
-      <c r="H36" s="29" t="s">
-        <v>121</v>
-      </c>
-      <c r="J36"/>
-    </row>
-    <row r="37" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A37" s="29" t="s">
-        <v>77</v>
-      </c>
-      <c r="B37" s="29" t="s">
-        <v>42</v>
-      </c>
-      <c r="C37" s="13"/>
-      <c r="D37" s="29" t="s">
-        <v>116</v>
-      </c>
-      <c r="E37" s="29" t="s">
-        <v>170</v>
-      </c>
-      <c r="F37" s="29" t="s">
-        <v>134</v>
-      </c>
-      <c r="G37" s="30" t="s">
-        <v>133</v>
-      </c>
-      <c r="H37" s="29" t="s">
-        <v>121</v>
-      </c>
-      <c r="J37"/>
-    </row>
-    <row r="38" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A38" s="29" t="s">
-        <v>78</v>
-      </c>
-      <c r="B38" s="29" t="s">
-        <v>42</v>
-      </c>
-      <c r="C38" s="13"/>
-      <c r="D38" s="29" t="s">
-        <v>117</v>
-      </c>
-      <c r="E38" s="29" t="s">
-        <v>171</v>
-      </c>
-      <c r="F38" s="29" t="s">
-        <v>134</v>
-      </c>
-      <c r="G38" s="30" t="s">
-        <v>133</v>
-      </c>
-      <c r="H38" s="29" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="39" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A39" s="29" t="s">
-        <v>79</v>
-      </c>
-      <c r="B39" s="29" t="s">
-        <v>42</v>
-      </c>
-      <c r="C39" s="13"/>
-      <c r="D39" s="29" t="s">
-        <v>118</v>
-      </c>
-      <c r="E39" s="29" t="s">
-        <v>172</v>
-      </c>
-      <c r="F39" s="29" t="s">
-        <v>134</v>
-      </c>
-      <c r="G39" s="30" t="s">
-        <v>133</v>
-      </c>
-      <c r="H39" s="29" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="40" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A40" s="29" t="s">
-        <v>80</v>
-      </c>
-      <c r="B40" s="29" t="s">
-        <v>42</v>
-      </c>
-      <c r="C40" s="13"/>
-      <c r="D40" s="29" t="s">
-        <v>119</v>
-      </c>
-      <c r="E40" s="29" t="s">
-        <v>173</v>
-      </c>
-      <c r="F40" s="29" t="s">
-        <v>134</v>
-      </c>
-      <c r="G40" s="30" t="s">
-        <v>133</v>
-      </c>
-      <c r="H40" s="29" t="s">
-        <v>124</v>
       </c>
     </row>
   </sheetData>
@@ -3347,322 +3420,331 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="26" t="s">
         <v>29</v>
       </c>
-      <c r="B1" s="28"/>
-      <c r="C1" s="28"/>
-      <c r="D1" s="28"/>
-      <c r="E1" s="28"/>
-      <c r="F1" s="28"/>
-      <c r="G1" s="28"/>
-      <c r="H1" s="28"/>
-      <c r="I1" s="28"/>
-      <c r="J1" s="28"/>
+      <c r="B1" s="26"/>
+      <c r="C1" s="26"/>
+      <c r="D1" s="26"/>
+      <c r="E1" s="26"/>
+      <c r="F1" s="26"/>
+      <c r="G1" s="26"/>
+      <c r="H1" s="26"/>
+      <c r="I1" s="26"/>
+      <c r="J1" s="26"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A2" s="28"/>
-      <c r="B2" s="28"/>
-      <c r="C2" s="28"/>
-      <c r="D2" s="28"/>
-      <c r="E2" s="28"/>
-      <c r="F2" s="28"/>
-      <c r="G2" s="28"/>
-      <c r="H2" s="28"/>
-      <c r="I2" s="28"/>
-      <c r="J2" s="28"/>
+      <c r="A2" s="26"/>
+      <c r="B2" s="26"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="26"/>
+      <c r="E2" s="26"/>
+      <c r="F2" s="26"/>
+      <c r="G2" s="26"/>
+      <c r="H2" s="26"/>
+      <c r="I2" s="26"/>
+      <c r="J2" s="26"/>
     </row>
     <row r="4" spans="1:10" ht="31" x14ac:dyDescent="0.35">
-      <c r="A4" s="26" t="s">
+      <c r="A4" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="B4" s="26" t="s">
+      <c r="B4" s="21" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="26" t="s">
+      <c r="C4" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="D4" s="26" t="s">
+      <c r="D4" s="21" t="s">
         <v>3</v>
       </c>
-      <c r="E4" s="26" t="s">
+      <c r="E4" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="F4" s="26" t="s">
+      <c r="F4" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="G4" s="26" t="s">
+      <c r="G4" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="H4" s="26" t="s">
+      <c r="H4" s="21" t="s">
         <v>7</v>
       </c>
-      <c r="I4" s="26" t="s">
+      <c r="I4" s="21" t="s">
         <v>30</v>
       </c>
-      <c r="J4" s="27" t="s">
+      <c r="J4" s="22" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="46.5" x14ac:dyDescent="0.35">
-      <c r="A5" s="15" t="s">
-        <v>37</v>
-      </c>
-      <c r="B5" s="15" t="s">
-        <v>36</v>
-      </c>
-      <c r="C5" s="15" t="s">
-        <v>31</v>
-      </c>
-      <c r="D5" s="15" t="s">
-        <v>32</v>
-      </c>
-      <c r="E5" s="16" t="s">
-        <v>33</v>
-      </c>
-      <c r="F5" s="15" t="s">
-        <v>34</v>
-      </c>
-      <c r="G5" s="15" t="s">
-        <v>35</v>
-      </c>
-      <c r="H5" s="17" t="s">
-        <v>40</v>
-      </c>
-      <c r="I5" s="18" t="s">
-        <v>38</v>
-      </c>
-      <c r="J5" s="19" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A6" s="20"/>
-      <c r="B6" s="20"/>
-      <c r="C6" s="20"/>
-      <c r="D6" s="20"/>
-      <c r="E6" s="20"/>
-      <c r="F6" s="20"/>
-      <c r="G6" s="20"/>
-      <c r="H6" s="20"/>
-      <c r="I6" s="21"/>
-      <c r="J6" s="22"/>
+    <row r="5" spans="1:10" ht="31" x14ac:dyDescent="0.35">
+      <c r="A5" s="35" t="s">
+        <v>166</v>
+      </c>
+      <c r="B5" s="30" t="s">
+        <v>33</v>
+      </c>
+      <c r="C5" s="36"/>
+      <c r="D5" s="35" t="s">
+        <v>165</v>
+      </c>
+      <c r="E5" s="28" t="s">
+        <v>171</v>
+      </c>
+      <c r="F5" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="G5" s="33" t="s">
+        <v>124</v>
+      </c>
+      <c r="H5" s="37" t="s">
+        <v>168</v>
+      </c>
+      <c r="I5" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="J5" s="14"/>
+    </row>
+    <row r="6" spans="1:10" ht="31" x14ac:dyDescent="0.35">
+      <c r="A6" s="35" t="s">
+        <v>167</v>
+      </c>
+      <c r="B6" s="30" t="s">
+        <v>33</v>
+      </c>
+      <c r="C6" s="36"/>
+      <c r="D6" s="37" t="s">
+        <v>164</v>
+      </c>
+      <c r="E6" s="36" t="s">
+        <v>170</v>
+      </c>
+      <c r="F6" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="G6" s="33" t="s">
+        <v>124</v>
+      </c>
+      <c r="H6" s="37" t="s">
+        <v>169</v>
+      </c>
+      <c r="I6" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="J6" s="17"/>
     </row>
     <row r="7" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A7" s="20"/>
-      <c r="B7" s="20"/>
-      <c r="C7" s="20"/>
-      <c r="D7" s="20"/>
-      <c r="E7" s="20"/>
-      <c r="F7" s="20"/>
-      <c r="G7" s="20"/>
-      <c r="H7" s="20"/>
-      <c r="I7" s="21"/>
-      <c r="J7" s="22"/>
+      <c r="A7" s="15"/>
+      <c r="B7" s="15"/>
+      <c r="C7" s="15"/>
+      <c r="D7" s="15"/>
+      <c r="E7" s="15"/>
+      <c r="F7" s="15"/>
+      <c r="G7" s="15"/>
+      <c r="H7" s="15"/>
+      <c r="I7" s="16"/>
+      <c r="J7" s="17"/>
     </row>
     <row r="8" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A8" s="20"/>
-      <c r="B8" s="20"/>
-      <c r="C8" s="20"/>
-      <c r="D8" s="20"/>
-      <c r="E8" s="20"/>
-      <c r="F8" s="20"/>
-      <c r="G8" s="20"/>
-      <c r="H8" s="20"/>
-      <c r="I8" s="21"/>
-      <c r="J8" s="22"/>
+      <c r="A8" s="15"/>
+      <c r="B8" s="15"/>
+      <c r="C8" s="15"/>
+      <c r="D8" s="15"/>
+      <c r="E8" s="15"/>
+      <c r="F8" s="15"/>
+      <c r="G8" s="15"/>
+      <c r="H8" s="15"/>
+      <c r="I8" s="16"/>
+      <c r="J8" s="17"/>
     </row>
     <row r="9" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A9" s="20"/>
-      <c r="B9" s="20"/>
-      <c r="C9" s="20"/>
-      <c r="D9" s="20"/>
-      <c r="E9" s="20"/>
-      <c r="F9" s="20"/>
-      <c r="G9" s="20"/>
-      <c r="H9" s="20"/>
-      <c r="I9" s="21"/>
-      <c r="J9" s="22"/>
+      <c r="A9" s="15"/>
+      <c r="B9" s="15"/>
+      <c r="C9" s="15"/>
+      <c r="D9" s="15"/>
+      <c r="E9" s="15"/>
+      <c r="F9" s="15"/>
+      <c r="G9" s="15"/>
+      <c r="H9" s="15"/>
+      <c r="I9" s="16"/>
+      <c r="J9" s="17"/>
     </row>
     <row r="10" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A10" s="20"/>
-      <c r="B10" s="20"/>
-      <c r="C10" s="20"/>
-      <c r="D10" s="20"/>
-      <c r="E10" s="20"/>
-      <c r="F10" s="20"/>
-      <c r="G10" s="20"/>
-      <c r="H10" s="20"/>
-      <c r="I10" s="21"/>
-      <c r="J10" s="22"/>
+      <c r="A10" s="15"/>
+      <c r="B10" s="15"/>
+      <c r="C10" s="15"/>
+      <c r="D10" s="15"/>
+      <c r="E10" s="15"/>
+      <c r="F10" s="15"/>
+      <c r="G10" s="15"/>
+      <c r="H10" s="15"/>
+      <c r="I10" s="16"/>
+      <c r="J10" s="17"/>
     </row>
     <row r="11" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A11" s="20"/>
-      <c r="B11" s="20"/>
-      <c r="C11" s="20"/>
-      <c r="D11" s="20"/>
-      <c r="E11" s="20"/>
-      <c r="F11" s="20"/>
-      <c r="G11" s="20"/>
-      <c r="H11" s="20"/>
-      <c r="I11" s="21"/>
-      <c r="J11" s="22"/>
+      <c r="A11" s="15"/>
+      <c r="B11" s="15"/>
+      <c r="C11" s="15"/>
+      <c r="D11" s="15"/>
+      <c r="E11" s="15"/>
+      <c r="F11" s="15"/>
+      <c r="G11" s="15"/>
+      <c r="H11" s="15"/>
+      <c r="I11" s="16"/>
+      <c r="J11" s="17"/>
     </row>
     <row r="12" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A12" s="20"/>
-      <c r="B12" s="20"/>
-      <c r="C12" s="20"/>
-      <c r="D12" s="20"/>
-      <c r="E12" s="20"/>
-      <c r="F12" s="20"/>
-      <c r="G12" s="20"/>
-      <c r="H12" s="20"/>
-      <c r="I12" s="21"/>
-      <c r="J12" s="22"/>
+      <c r="A12" s="15"/>
+      <c r="B12" s="15"/>
+      <c r="C12" s="15"/>
+      <c r="D12" s="15"/>
+      <c r="E12" s="15"/>
+      <c r="F12" s="15"/>
+      <c r="G12" s="15"/>
+      <c r="H12" s="15"/>
+      <c r="I12" s="16"/>
+      <c r="J12" s="17"/>
     </row>
     <row r="13" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A13" s="20"/>
-      <c r="B13" s="20"/>
-      <c r="C13" s="20"/>
-      <c r="D13" s="20"/>
-      <c r="E13" s="20"/>
-      <c r="F13" s="20"/>
-      <c r="G13" s="20"/>
-      <c r="H13" s="20"/>
-      <c r="I13" s="21"/>
-      <c r="J13" s="22"/>
+      <c r="A13" s="15"/>
+      <c r="B13" s="15"/>
+      <c r="C13" s="15"/>
+      <c r="D13" s="15"/>
+      <c r="E13" s="15"/>
+      <c r="F13" s="15"/>
+      <c r="G13" s="15"/>
+      <c r="H13" s="15"/>
+      <c r="I13" s="16"/>
+      <c r="J13" s="17"/>
     </row>
     <row r="14" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A14" s="20"/>
-      <c r="B14" s="20"/>
-      <c r="C14" s="20"/>
-      <c r="D14" s="20"/>
-      <c r="E14" s="20"/>
-      <c r="F14" s="20"/>
-      <c r="G14" s="20"/>
-      <c r="H14" s="20"/>
-      <c r="I14" s="21"/>
-      <c r="J14" s="22"/>
+      <c r="A14" s="15"/>
+      <c r="B14" s="15"/>
+      <c r="C14" s="15"/>
+      <c r="D14" s="15"/>
+      <c r="E14" s="15"/>
+      <c r="F14" s="15"/>
+      <c r="G14" s="15"/>
+      <c r="H14" s="15"/>
+      <c r="I14" s="16"/>
+      <c r="J14" s="17"/>
     </row>
     <row r="15" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A15" s="20"/>
-      <c r="B15" s="20"/>
-      <c r="C15" s="20"/>
-      <c r="D15" s="20"/>
-      <c r="E15" s="20"/>
-      <c r="F15" s="20"/>
-      <c r="G15" s="20"/>
-      <c r="H15" s="20"/>
-      <c r="I15" s="21"/>
-      <c r="J15" s="22"/>
+      <c r="A15" s="15"/>
+      <c r="B15" s="15"/>
+      <c r="C15" s="15"/>
+      <c r="D15" s="15"/>
+      <c r="E15" s="15"/>
+      <c r="F15" s="15"/>
+      <c r="G15" s="15"/>
+      <c r="H15" s="15"/>
+      <c r="I15" s="16"/>
+      <c r="J15" s="17"/>
     </row>
     <row r="16" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A16" s="20"/>
-      <c r="B16" s="20"/>
-      <c r="C16" s="20"/>
-      <c r="D16" s="20"/>
-      <c r="E16" s="20"/>
-      <c r="F16" s="20"/>
-      <c r="G16" s="20"/>
-      <c r="H16" s="20"/>
-      <c r="I16" s="21"/>
-      <c r="J16" s="22"/>
+      <c r="A16" s="15"/>
+      <c r="B16" s="15"/>
+      <c r="C16" s="15"/>
+      <c r="D16" s="15"/>
+      <c r="E16" s="15"/>
+      <c r="F16" s="15"/>
+      <c r="G16" s="15"/>
+      <c r="H16" s="15"/>
+      <c r="I16" s="16"/>
+      <c r="J16" s="17"/>
     </row>
     <row r="17" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A17" s="20"/>
-      <c r="B17" s="20"/>
-      <c r="C17" s="20"/>
-      <c r="D17" s="20"/>
-      <c r="E17" s="20"/>
-      <c r="F17" s="20"/>
-      <c r="G17" s="20"/>
-      <c r="H17" s="20"/>
-      <c r="I17" s="21"/>
-      <c r="J17" s="22"/>
+      <c r="A17" s="15"/>
+      <c r="B17" s="15"/>
+      <c r="C17" s="15"/>
+      <c r="D17" s="15"/>
+      <c r="E17" s="15"/>
+      <c r="F17" s="15"/>
+      <c r="G17" s="15"/>
+      <c r="H17" s="15"/>
+      <c r="I17" s="16"/>
+      <c r="J17" s="17"/>
     </row>
     <row r="18" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A18" s="20"/>
-      <c r="B18" s="20"/>
-      <c r="C18" s="20"/>
-      <c r="D18" s="20"/>
-      <c r="E18" s="20"/>
-      <c r="F18" s="20"/>
-      <c r="G18" s="20"/>
-      <c r="H18" s="20"/>
-      <c r="I18" s="21"/>
-      <c r="J18" s="22"/>
+      <c r="A18" s="15"/>
+      <c r="B18" s="15"/>
+      <c r="C18" s="15"/>
+      <c r="D18" s="15"/>
+      <c r="E18" s="15"/>
+      <c r="F18" s="15"/>
+      <c r="G18" s="15"/>
+      <c r="H18" s="15"/>
+      <c r="I18" s="16"/>
+      <c r="J18" s="17"/>
     </row>
     <row r="19" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A19" s="20"/>
-      <c r="B19" s="20"/>
-      <c r="C19" s="20"/>
-      <c r="D19" s="20"/>
-      <c r="E19" s="20"/>
-      <c r="F19" s="20"/>
-      <c r="G19" s="20"/>
-      <c r="H19" s="20"/>
-      <c r="I19" s="21"/>
-      <c r="J19" s="22"/>
+      <c r="A19" s="15"/>
+      <c r="B19" s="15"/>
+      <c r="C19" s="15"/>
+      <c r="D19" s="15"/>
+      <c r="E19" s="15"/>
+      <c r="F19" s="15"/>
+      <c r="G19" s="15"/>
+      <c r="H19" s="15"/>
+      <c r="I19" s="16"/>
+      <c r="J19" s="17"/>
     </row>
     <row r="20" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A20" s="20"/>
-      <c r="B20" s="20"/>
-      <c r="C20" s="20"/>
-      <c r="D20" s="20"/>
-      <c r="E20" s="20"/>
-      <c r="F20" s="20"/>
-      <c r="G20" s="20"/>
-      <c r="H20" s="20"/>
-      <c r="I20" s="21"/>
-      <c r="J20" s="22"/>
+      <c r="A20" s="15"/>
+      <c r="B20" s="15"/>
+      <c r="C20" s="15"/>
+      <c r="D20" s="15"/>
+      <c r="E20" s="15"/>
+      <c r="F20" s="15"/>
+      <c r="G20" s="15"/>
+      <c r="H20" s="15"/>
+      <c r="I20" s="16"/>
+      <c r="J20" s="17"/>
     </row>
     <row r="21" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A21" s="20"/>
-      <c r="B21" s="20"/>
-      <c r="C21" s="20"/>
-      <c r="D21" s="20"/>
-      <c r="E21" s="20"/>
-      <c r="F21" s="20"/>
-      <c r="G21" s="20"/>
-      <c r="H21" s="20"/>
-      <c r="I21" s="21"/>
-      <c r="J21" s="22"/>
+      <c r="A21" s="15"/>
+      <c r="B21" s="15"/>
+      <c r="C21" s="15"/>
+      <c r="D21" s="15"/>
+      <c r="E21" s="15"/>
+      <c r="F21" s="15"/>
+      <c r="G21" s="15"/>
+      <c r="H21" s="15"/>
+      <c r="I21" s="16"/>
+      <c r="J21" s="17"/>
     </row>
     <row r="22" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A22" s="20"/>
-      <c r="B22" s="20"/>
-      <c r="C22" s="20"/>
-      <c r="D22" s="20"/>
-      <c r="E22" s="20"/>
-      <c r="F22" s="20"/>
-      <c r="G22" s="20"/>
-      <c r="H22" s="20"/>
-      <c r="I22" s="21"/>
-      <c r="J22" s="22"/>
+      <c r="A22" s="15"/>
+      <c r="B22" s="15"/>
+      <c r="C22" s="15"/>
+      <c r="D22" s="15"/>
+      <c r="E22" s="15"/>
+      <c r="F22" s="15"/>
+      <c r="G22" s="15"/>
+      <c r="H22" s="15"/>
+      <c r="I22" s="16"/>
+      <c r="J22" s="17"/>
     </row>
     <row r="23" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A23" s="23"/>
-      <c r="B23" s="23"/>
-      <c r="C23" s="23"/>
-      <c r="D23" s="23"/>
-      <c r="E23" s="23"/>
-      <c r="F23" s="23"/>
-      <c r="G23" s="23"/>
-      <c r="H23" s="23"/>
-      <c r="I23" s="24"/>
-      <c r="J23" s="25"/>
+      <c r="A23" s="18"/>
+      <c r="B23" s="18"/>
+      <c r="C23" s="18"/>
+      <c r="D23" s="18"/>
+      <c r="E23" s="18"/>
+      <c r="F23" s="18"/>
+      <c r="G23" s="18"/>
+      <c r="H23" s="18"/>
+      <c r="I23" s="19"/>
+      <c r="J23" s="20"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:J2"/>
   </mergeCells>
-  <hyperlinks>
-    <hyperlink ref="E5" r:id="rId1" xr:uid="{A941C51A-735A-424E-9F09-945F539595B9}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId2"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId3"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
@@ -3726,7 +3808,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" s="5" t="s">
-        <v>41</v>
+        <v>32</v>
       </c>
       <c r="B7" s="6" t="s">
         <v>21</v>

</xml_diff>